<commit_message>
feature/fsel-5726: Update Code Export File SummaryReport
</commit_message>
<xml_diff>
--- a/Services/Fsel.Course/Fsel.Course.Lcms.Api/Resources/ExportExcelTemplates/BaoCao_CapPhong.xlsx
+++ b/Services/Fsel.Course/Fsel.Course.Lcms.Api/Resources/ExportExcelTemplates/BaoCao_CapPhong.xlsx
@@ -1,15 +1,16 @@
 
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
-<workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" mc:Ignorable="x15">
-  <fileVersion appName="xl" lastEdited="6" lowestEdited="6" rupBuild="14420"/>
-  <workbookPr/>
+<workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr6="http://schemas.microsoft.com/office/spreadsheetml/2016/revision6" xmlns:xr10="http://schemas.microsoft.com/office/spreadsheetml/2016/revision10" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" mc:Ignorable="x15 xr xr6 xr10 xr2">
+  <fileVersion appName="xl" lastEdited="7" lowestEdited="7" rupBuild="28827"/>
+  <workbookPr defaultThemeVersion="166925"/>
   <mc:AlternateContent xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
     <mc:Choice Requires="x15">
-      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Code\FSEL_All\Fsel\fsel_src\Services\Fsel.Course\Fsel.Course.Lcms.Api\Resources\ExportExcelTemplates\"/>
+      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="D:\PhanPhuc\Fsel\fsel_src\Services\Fsel.Course\Fsel.Course.Lcms.Api\Resources\ExportExcelTemplates\"/>
     </mc:Choice>
   </mc:AlternateContent>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{5C422327-C22C-427B-9987-468BF9ACEB47}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="0" yWindow="0" windowWidth="15870" windowHeight="12045"/>
+    <workbookView xWindow="-28920" yWindow="-120" windowWidth="29040" windowHeight="15720" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
   <sheets>
     <sheet name="Sheet1" sheetId="1" r:id="rId1"/>
@@ -24,7 +25,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="16" uniqueCount="16">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="64" uniqueCount="52">
   <si>
     <t>BÁO CÁO GIAI ĐOẠN ĐĂNG KÝ "THÁNG TỰ HỌC TIẾNG ANH"</t>
   </si>
@@ -74,17 +75,126 @@
   </si>
   <si>
     <t>THCS</t>
+  </si>
+  <si>
+    <t>BÁO CÁO XÁC THỰC</t>
+  </si>
+  <si>
+    <t>BÁO CÁO ĐÁNH GIÁ ĐẦU VÀO (PT)</t>
+  </si>
+  <si>
+    <t>BÁO CÁO VÀO HỌC</t>
+  </si>
+  <si>
+    <t>Số HS xác thực thành công</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Tỷ lệ HS xác thực thành công/SL thực tế </t>
+  </si>
+  <si>
+    <t>Số lượng GV xác thực thành công</t>
+  </si>
+  <si>
+    <t xml:space="preserve">tỷ lệ GV xác thực thành công/ SL thực tế </t>
+  </si>
+  <si>
+    <t>Tổng số Học viên xác thực
+(HS+GV)</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Tỷ lệ học viên xác thực tham gia/SL thực tế </t>
+  </si>
+  <si>
+    <t>HỌC SINH</t>
+  </si>
+  <si>
+    <t>GIÁO VIÊN</t>
+  </si>
+  <si>
+    <t>HỌC VIÊN</t>
+  </si>
+  <si>
+    <t>Số HS đã học trên hệ thống</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Tỷ lệ HS đã học/SL thực tế </t>
+  </si>
+  <si>
+    <t>Số GV đã học trên hệ thống</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Tỷ lệ GV đã học/SL thực tế </t>
+  </si>
+  <si>
+    <t>Số Học viên (HS+GV) đã học trên hệ thống</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Tỷ lệ học viên đã học/SL thực tế </t>
+  </si>
+  <si>
+    <t>SL HS đã hoàn thành PT</t>
+  </si>
+  <si>
+    <t>Tỷ lệ HS hoàn thành PT/SL đăng ký</t>
+  </si>
+  <si>
+    <t>Tỷ lệ HS hoàn thành PT/SL thực tế</t>
+  </si>
+  <si>
+    <t>SL HS đang PT</t>
+  </si>
+  <si>
+    <t>Tỷ lệ HS đang PT/SL đăng ký</t>
+  </si>
+  <si>
+    <t>Tỷ lệ HS đang PT/SL thực tế</t>
+  </si>
+  <si>
+    <t>SL GV đã hoàn thành PT</t>
+  </si>
+  <si>
+    <t>Tỷ lệ GV hoàn thành PT/SL đăng ký</t>
+  </si>
+  <si>
+    <t>Tỷ lệ GV hoàn thành PT/SL thực tế</t>
+  </si>
+  <si>
+    <t>SL GV đang PT</t>
+  </si>
+  <si>
+    <t>Tỷ lệ GV đang PT/SL đăng ký</t>
+  </si>
+  <si>
+    <t>Tỷ lệ GV đang PT/SL thực tế</t>
+  </si>
+  <si>
+    <t>SL HV đã hoàn thành PT</t>
+  </si>
+  <si>
+    <t>Tỷ lệ HV hoàn thành PT/SL đăng ký</t>
+  </si>
+  <si>
+    <t>Tỷ lệ HV hoàn thành PT/SL thực tế</t>
+  </si>
+  <si>
+    <t>SL HV đang PT</t>
+  </si>
+  <si>
+    <t>Tỷ lệ HV đang PT/SL đăng ký</t>
+  </si>
+  <si>
+    <t>Tỷ lệ HV đang PT/SL thực tế</t>
   </si>
 </sst>
 </file>
 
 <file path=xl/styles.xml><?xml version="1.0" encoding="utf-8"?>
-<styleSheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:x16r2="http://schemas.microsoft.com/office/spreadsheetml/2015/02/main" mc:Ignorable="x14ac x16r2">
+<styleSheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:x16r2="http://schemas.microsoft.com/office/spreadsheetml/2015/02/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" mc:Ignorable="x14ac x16r2 xr">
   <fonts count="7" x14ac:knownFonts="1">
     <font>
       <sz val="11"/>
       <color theme="1"/>
-      <name val="Calibri"/>
+      <name val="Arial"/>
       <family val="2"/>
       <scheme val="minor"/>
     </font>
@@ -92,7 +202,7 @@
       <b/>
       <sz val="11"/>
       <color theme="1"/>
-      <name val="Calibri"/>
+      <name val="Arial"/>
       <family val="2"/>
       <scheme val="minor"/>
     </font>
@@ -100,7 +210,7 @@
       <b/>
       <sz val="18"/>
       <color theme="1"/>
-      <name val="Calibri"/>
+      <name val="Arial"/>
       <family val="2"/>
       <scheme val="minor"/>
     </font>
@@ -108,7 +218,7 @@
       <b/>
       <sz val="20"/>
       <color theme="1"/>
-      <name val="Calibri"/>
+      <name val="Arial"/>
       <family val="2"/>
       <scheme val="minor"/>
     </font>
@@ -116,7 +226,7 @@
       <b/>
       <sz val="12"/>
       <color theme="1"/>
-      <name val="Calibri"/>
+      <name val="Arial"/>
       <family val="2"/>
       <scheme val="minor"/>
     </font>
@@ -124,19 +234,19 @@
       <b/>
       <sz val="15"/>
       <color theme="1"/>
-      <name val="Calibri"/>
+      <name val="Arial"/>
       <family val="2"/>
       <scheme val="minor"/>
     </font>
     <font>
       <sz val="15"/>
       <color theme="1"/>
-      <name val="Calibri"/>
+      <name val="Arial"/>
       <family val="2"/>
       <scheme val="minor"/>
     </font>
   </fonts>
-  <fills count="5">
+  <fills count="7">
     <fill>
       <patternFill patternType="none"/>
     </fill>
@@ -161,25 +271,24 @@
         <bgColor indexed="64"/>
       </patternFill>
     </fill>
+    <fill>
+      <patternFill patternType="solid">
+        <fgColor theme="6" tint="0.39997558519241921"/>
+        <bgColor indexed="64"/>
+      </patternFill>
+    </fill>
+    <fill>
+      <patternFill patternType="solid">
+        <fgColor theme="7" tint="0.79998168889431442"/>
+        <bgColor indexed="64"/>
+      </patternFill>
+    </fill>
   </fills>
-  <borders count="3">
+  <borders count="2">
     <border>
       <left/>
       <right/>
       <top/>
-      <bottom/>
-      <diagonal/>
-    </border>
-    <border>
-      <left style="thin">
-        <color rgb="FF000000"/>
-      </left>
-      <right style="thin">
-        <color rgb="FF000000"/>
-      </right>
-      <top style="thin">
-        <color rgb="FF000000"/>
-      </top>
       <bottom/>
       <diagonal/>
     </border>
@@ -202,7 +311,7 @@
   <cellStyleXfs count="1">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
   </cellStyleXfs>
-  <cellXfs count="13">
+  <cellXfs count="15">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0"/>
     <xf numFmtId="0" fontId="2" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
       <alignment horizontal="left"/>
@@ -217,10 +326,7 @@
     <xf numFmtId="0" fontId="6" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
       <alignment wrapText="1"/>
     </xf>
-    <xf numFmtId="0" fontId="1" fillId="0" borderId="2" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="1" fillId="4" borderId="2" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+    <xf numFmtId="0" fontId="1" fillId="0" borderId="1" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center" wrapText="1"/>
     </xf>
     <xf numFmtId="0" fontId="1" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
@@ -229,13 +335,22 @@
     <xf numFmtId="0" fontId="1" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
       <alignment horizontal="left" vertical="center" wrapText="1"/>
     </xf>
-    <xf numFmtId="0" fontId="0" fillId="4" borderId="0" xfId="0" applyFill="1" applyAlignment="1">
-      <alignment wrapText="1"/>
+    <xf numFmtId="0" fontId="1" fillId="0" borderId="1" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="1" fillId="4" borderId="1" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="5" fillId="6" borderId="1" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" wrapText="1"/>
     </xf>
     <xf numFmtId="0" fontId="5" fillId="2" borderId="1" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" wrapText="1"/>
     </xf>
     <xf numFmtId="0" fontId="5" fillId="3" borderId="1" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="5" fillId="5" borderId="1" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" wrapText="1"/>
     </xf>
   </cellXfs>
@@ -551,96 +666,323 @@
 </file>
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
-<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" mc:Ignorable="x14ac">
-  <dimension ref="A1:K14"/>
-  <sheetFormatPr defaultColWidth="18.7109375" defaultRowHeight="15" x14ac:dyDescent="0.25"/>
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{00000000-0001-0000-0000-000000000000}">
+  <dimension ref="A1:AO10"/>
+  <sheetFormatPr defaultColWidth="18.75" defaultRowHeight="14.25" x14ac:dyDescent="0.2"/>
   <cols>
-    <col min="1" max="1" width="14.85546875" style="2" customWidth="1"/>
-    <col min="2" max="2" width="20.5703125" style="2" customWidth="1"/>
-    <col min="3" max="5" width="18.28515625" style="2" customWidth="1"/>
-    <col min="6" max="11" width="20.85546875" style="2" customWidth="1"/>
-    <col min="12" max="16384" width="18.7109375" style="2"/>
+    <col min="1" max="1" width="14.875" style="2" customWidth="1"/>
+    <col min="2" max="2" width="20.625" style="2" customWidth="1"/>
+    <col min="3" max="5" width="18.25" style="2" customWidth="1"/>
+    <col min="6" max="11" width="20.875" style="2" customWidth="1"/>
+    <col min="12" max="16384" width="18.75" style="2"/>
   </cols>
   <sheetData>
-    <row r="1" spans="1:11" ht="26.25" x14ac:dyDescent="0.4">
+    <row r="1" spans="1:41" ht="26.25" x14ac:dyDescent="0.4">
       <c r="A1" s="1" t="s">
         <v>0</v>
       </c>
       <c r="F1" s="3"/>
     </row>
-    <row r="2" spans="1:11" ht="26.25" x14ac:dyDescent="0.4">
+    <row r="2" spans="1:41" ht="26.25" x14ac:dyDescent="0.4">
       <c r="A2" s="4" t="s">
         <v>13</v>
       </c>
       <c r="F2" s="3"/>
     </row>
-    <row r="3" spans="1:11" ht="26.25" x14ac:dyDescent="0.4">
+    <row r="3" spans="1:41" ht="26.25" x14ac:dyDescent="0.4">
       <c r="A3" s="4" t="s">
         <v>1</v>
       </c>
       <c r="F3" s="3"/>
     </row>
-    <row r="4" spans="1:11" s="5" customFormat="1" ht="19.5" x14ac:dyDescent="0.3">
-      <c r="A4" s="11" t="s">
+    <row r="4" spans="1:41" s="5" customFormat="1" ht="19.5" x14ac:dyDescent="0.3">
+      <c r="A4" s="12" t="s">
         <v>2</v>
       </c>
-      <c r="B4" s="11"/>
-      <c r="C4" s="11"/>
-      <c r="D4" s="11"/>
-      <c r="E4" s="11"/>
-      <c r="F4" s="12" t="s">
+      <c r="B4" s="12"/>
+      <c r="C4" s="12"/>
+      <c r="D4" s="12"/>
+      <c r="E4" s="12"/>
+      <c r="F4" s="13" t="s">
         <v>14</v>
       </c>
-      <c r="G4" s="12"/>
-      <c r="H4" s="12"/>
-      <c r="I4" s="12"/>
-      <c r="J4" s="12"/>
-      <c r="K4" s="12"/>
+      <c r="G4" s="13"/>
+      <c r="H4" s="13"/>
+      <c r="I4" s="13"/>
+      <c r="J4" s="13"/>
+      <c r="K4" s="13"/>
+      <c r="L4" s="14" t="s">
+        <v>16</v>
+      </c>
+      <c r="M4" s="14"/>
+      <c r="N4" s="14"/>
+      <c r="O4" s="14"/>
+      <c r="P4" s="14"/>
+      <c r="Q4" s="14"/>
+      <c r="R4" s="11" t="s">
+        <v>17</v>
+      </c>
+      <c r="S4" s="11"/>
+      <c r="T4" s="11"/>
+      <c r="U4" s="11"/>
+      <c r="V4" s="11"/>
+      <c r="W4" s="11"/>
+      <c r="X4" s="11"/>
+      <c r="Y4" s="11"/>
+      <c r="Z4" s="11"/>
+      <c r="AA4" s="11"/>
+      <c r="AB4" s="11"/>
+      <c r="AC4" s="11"/>
+      <c r="AD4" s="11"/>
+      <c r="AE4" s="11"/>
+      <c r="AF4" s="11"/>
+      <c r="AG4" s="11"/>
+      <c r="AH4" s="11"/>
+      <c r="AI4" s="11"/>
+      <c r="AJ4" s="14" t="s">
+        <v>18</v>
+      </c>
+      <c r="AK4" s="14"/>
+      <c r="AL4" s="14"/>
+      <c r="AM4" s="14"/>
+      <c r="AN4" s="14"/>
+      <c r="AO4" s="14"/>
     </row>
-    <row r="5" spans="1:11" s="8" customFormat="1" ht="45" x14ac:dyDescent="0.25">
-      <c r="A5" s="6"/>
-      <c r="B5" s="6" t="s">
+    <row r="5" spans="1:41" s="7" customFormat="1" ht="45" customHeight="1" x14ac:dyDescent="0.3">
+      <c r="A5" s="9"/>
+      <c r="B5" s="9" t="s">
         <v>3</v>
       </c>
-      <c r="C5" s="6" t="s">
+      <c r="C5" s="9" t="s">
         <v>4</v>
       </c>
-      <c r="D5" s="6" t="s">
+      <c r="D5" s="9" t="s">
         <v>5</v>
       </c>
-      <c r="E5" s="6" t="s">
+      <c r="E5" s="9" t="s">
         <v>6</v>
       </c>
-      <c r="F5" s="7" t="s">
+      <c r="F5" s="10" t="s">
         <v>7</v>
       </c>
-      <c r="G5" s="7" t="s">
+      <c r="G5" s="10" t="s">
         <v>8</v>
       </c>
-      <c r="H5" s="7" t="s">
+      <c r="H5" s="10" t="s">
         <v>9</v>
       </c>
-      <c r="I5" s="7" t="s">
+      <c r="I5" s="10" t="s">
         <v>10</v>
       </c>
-      <c r="J5" s="6" t="s">
+      <c r="J5" s="9" t="s">
         <v>11</v>
       </c>
-      <c r="K5" s="7" t="s">
+      <c r="K5" s="10" t="s">
         <v>12</v>
       </c>
+      <c r="L5" s="9" t="s">
+        <v>19</v>
+      </c>
+      <c r="M5" s="9" t="s">
+        <v>20</v>
+      </c>
+      <c r="N5" s="9" t="s">
+        <v>21</v>
+      </c>
+      <c r="O5" s="9" t="s">
+        <v>22</v>
+      </c>
+      <c r="P5" s="9" t="s">
+        <v>23</v>
+      </c>
+      <c r="Q5" s="9" t="s">
+        <v>24</v>
+      </c>
+      <c r="R5" s="11" t="s">
+        <v>25</v>
+      </c>
+      <c r="S5" s="11"/>
+      <c r="T5" s="11"/>
+      <c r="U5" s="11"/>
+      <c r="V5" s="11"/>
+      <c r="W5" s="11"/>
+      <c r="X5" s="11" t="s">
+        <v>26</v>
+      </c>
+      <c r="Y5" s="11"/>
+      <c r="Z5" s="11"/>
+      <c r="AA5" s="11"/>
+      <c r="AB5" s="11"/>
+      <c r="AC5" s="11"/>
+      <c r="AD5" s="11" t="s">
+        <v>27</v>
+      </c>
+      <c r="AE5" s="11"/>
+      <c r="AF5" s="11"/>
+      <c r="AG5" s="11"/>
+      <c r="AH5" s="11"/>
+      <c r="AI5" s="11"/>
+      <c r="AJ5" s="9" t="s">
+        <v>28</v>
+      </c>
+      <c r="AK5" s="9" t="s">
+        <v>29</v>
+      </c>
+      <c r="AL5" s="9" t="s">
+        <v>30</v>
+      </c>
+      <c r="AM5" s="9" t="s">
+        <v>31</v>
+      </c>
+      <c r="AN5" s="9" t="s">
+        <v>32</v>
+      </c>
+      <c r="AO5" s="9" t="s">
+        <v>33</v>
+      </c>
     </row>
-    <row r="6" spans="1:11" s="9" customFormat="1" x14ac:dyDescent="0.25">
-      <c r="A6" s="9" t="s">
+    <row r="6" spans="1:41" s="8" customFormat="1" ht="45" x14ac:dyDescent="0.2">
+      <c r="A6" s="9"/>
+      <c r="B6" s="9"/>
+      <c r="C6" s="9"/>
+      <c r="D6" s="9"/>
+      <c r="E6" s="9"/>
+      <c r="F6" s="10"/>
+      <c r="G6" s="10"/>
+      <c r="H6" s="10"/>
+      <c r="I6" s="10"/>
+      <c r="J6" s="9"/>
+      <c r="K6" s="10"/>
+      <c r="L6" s="9" t="s">
+        <v>19</v>
+      </c>
+      <c r="M6" s="9" t="s">
+        <v>20</v>
+      </c>
+      <c r="N6" s="9" t="s">
+        <v>21</v>
+      </c>
+      <c r="O6" s="9" t="s">
+        <v>22</v>
+      </c>
+      <c r="P6" s="9" t="s">
+        <v>23</v>
+      </c>
+      <c r="Q6" s="9" t="s">
+        <v>24</v>
+      </c>
+      <c r="R6" s="6" t="s">
+        <v>34</v>
+      </c>
+      <c r="S6" s="6" t="s">
+        <v>35</v>
+      </c>
+      <c r="T6" s="6" t="s">
+        <v>36</v>
+      </c>
+      <c r="U6" s="6" t="s">
+        <v>37</v>
+      </c>
+      <c r="V6" s="6" t="s">
+        <v>38</v>
+      </c>
+      <c r="W6" s="6" t="s">
+        <v>39</v>
+      </c>
+      <c r="X6" s="6" t="s">
+        <v>40</v>
+      </c>
+      <c r="Y6" s="6" t="s">
+        <v>41</v>
+      </c>
+      <c r="Z6" s="6" t="s">
+        <v>42</v>
+      </c>
+      <c r="AA6" s="6" t="s">
+        <v>43</v>
+      </c>
+      <c r="AB6" s="6" t="s">
+        <v>44</v>
+      </c>
+      <c r="AC6" s="6" t="s">
+        <v>45</v>
+      </c>
+      <c r="AD6" s="6" t="s">
+        <v>46</v>
+      </c>
+      <c r="AE6" s="6" t="s">
+        <v>47</v>
+      </c>
+      <c r="AF6" s="6" t="s">
+        <v>48</v>
+      </c>
+      <c r="AG6" s="6" t="s">
+        <v>49</v>
+      </c>
+      <c r="AH6" s="6" t="s">
+        <v>50</v>
+      </c>
+      <c r="AI6" s="6" t="s">
+        <v>51</v>
+      </c>
+      <c r="AJ6" s="9" t="s">
+        <v>19</v>
+      </c>
+      <c r="AK6" s="9" t="s">
+        <v>20</v>
+      </c>
+      <c r="AL6" s="9" t="s">
+        <v>19</v>
+      </c>
+      <c r="AM6" s="9" t="s">
+        <v>20</v>
+      </c>
+      <c r="AN6" s="9" t="s">
+        <v>19</v>
+      </c>
+      <c r="AO6" s="9" t="s">
+        <v>20</v>
+      </c>
+    </row>
+    <row r="7" spans="1:41" ht="15" x14ac:dyDescent="0.2">
+      <c r="A7" s="8" t="s">
         <v>15</v>
       </c>
     </row>
-    <row r="10" spans="1:11" ht="15" customHeight="1" x14ac:dyDescent="0.25"/>
-    <row r="14" spans="1:11" s="10" customFormat="1" x14ac:dyDescent="0.25"/>
+    <row r="10" spans="1:41" ht="15" customHeight="1" x14ac:dyDescent="0.2"/>
   </sheetData>
-  <mergeCells count="2">
+  <mergeCells count="31">
     <mergeCell ref="A4:E4"/>
     <mergeCell ref="F4:K4"/>
+    <mergeCell ref="L4:Q4"/>
+    <mergeCell ref="R4:AI4"/>
+    <mergeCell ref="AJ4:AO4"/>
+    <mergeCell ref="AM5:AM6"/>
+    <mergeCell ref="AN5:AN6"/>
+    <mergeCell ref="AO5:AO6"/>
+    <mergeCell ref="O5:O6"/>
+    <mergeCell ref="P5:P6"/>
+    <mergeCell ref="Q5:Q6"/>
+    <mergeCell ref="R5:W5"/>
+    <mergeCell ref="X5:AC5"/>
+    <mergeCell ref="AD5:AI5"/>
+    <mergeCell ref="AJ5:AJ6"/>
+    <mergeCell ref="AK5:AK6"/>
+    <mergeCell ref="AL5:AL6"/>
+    <mergeCell ref="L5:L6"/>
+    <mergeCell ref="M5:M6"/>
+    <mergeCell ref="N5:N6"/>
+    <mergeCell ref="A5:A6"/>
+    <mergeCell ref="B5:B6"/>
+    <mergeCell ref="C5:C6"/>
+    <mergeCell ref="D5:D6"/>
+    <mergeCell ref="E5:E6"/>
+    <mergeCell ref="F5:F6"/>
+    <mergeCell ref="G5:G6"/>
+    <mergeCell ref="H5:H6"/>
+    <mergeCell ref="I5:I6"/>
+    <mergeCell ref="J5:J6"/>
+    <mergeCell ref="K5:K6"/>
   </mergeCells>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
 </worksheet>

</xml_diff>

<commit_message>
feature/fsel-5726: Update File Export Data BaoCao
</commit_message>
<xml_diff>
--- a/Services/Fsel.Course/Fsel.Course.Lcms.Api/Resources/ExportExcelTemplates/BaoCao_CapPhong.xlsx
+++ b/Services/Fsel.Course/Fsel.Course.Lcms.Api/Resources/ExportExcelTemplates/BaoCao_CapPhong.xlsx
@@ -8,7 +8,7 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="D:\PhanPhuc\Fsel\fsel_src\Services\Fsel.Course\Fsel.Course.Lcms.Api\Resources\ExportExcelTemplates\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{5C422327-C22C-427B-9987-468BF9ACEB47}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{A3BE6C73-B387-49D3-8256-302039FFB888}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
     <workbookView xWindow="-28920" yWindow="-120" windowWidth="29040" windowHeight="15720" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
@@ -27,9 +27,6 @@
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
 <sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="64" uniqueCount="52">
   <si>
-    <t>BÁO CÁO GIAI ĐOẠN ĐĂNG KÝ "THÁNG TỰ HỌC TIẾNG ANH"</t>
-  </si>
-  <si>
     <t>Ngày xuất báo cáo:</t>
   </si>
   <si>
@@ -184,6 +181,9 @@
   </si>
   <si>
     <t>Tỷ lệ HV đang PT/SL thực tế</t>
+  </si>
+  <si>
+    <t>BÁO CÁO HỌC TẬP "THÁNG TỰ HỌC TIẾNG ANH"</t>
   </si>
 </sst>
 </file>
@@ -335,15 +335,6 @@
     <xf numFmtId="0" fontId="1" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
       <alignment horizontal="left" vertical="center" wrapText="1"/>
     </xf>
-    <xf numFmtId="0" fontId="1" fillId="0" borderId="1" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="1" fillId="4" borderId="1" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="5" fillId="6" borderId="1" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" wrapText="1"/>
-    </xf>
     <xf numFmtId="0" fontId="5" fillId="2" borderId="1" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" wrapText="1"/>
     </xf>
@@ -352,6 +343,15 @@
     </xf>
     <xf numFmtId="0" fontId="5" fillId="5" borderId="1" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="5" fillId="6" borderId="1" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="1" fillId="0" borderId="1" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="1" fillId="4" borderId="1" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
     </xf>
   </cellXfs>
   <cellStyles count="1">
@@ -679,296 +679,279 @@
   <sheetData>
     <row r="1" spans="1:41" ht="26.25" x14ac:dyDescent="0.4">
       <c r="A1" s="1" t="s">
-        <v>0</v>
+        <v>51</v>
       </c>
       <c r="F1" s="3"/>
     </row>
     <row r="2" spans="1:41" ht="26.25" x14ac:dyDescent="0.4">
       <c r="A2" s="4" t="s">
-        <v>13</v>
+        <v>12</v>
       </c>
       <c r="F2" s="3"/>
     </row>
     <row r="3" spans="1:41" ht="26.25" x14ac:dyDescent="0.4">
       <c r="A3" s="4" t="s">
-        <v>1</v>
+        <v>0</v>
       </c>
       <c r="F3" s="3"/>
     </row>
     <row r="4" spans="1:41" s="5" customFormat="1" ht="19.5" x14ac:dyDescent="0.3">
-      <c r="A4" s="12" t="s">
-        <v>2</v>
-      </c>
-      <c r="B4" s="12"/>
-      <c r="C4" s="12"/>
-      <c r="D4" s="12"/>
-      <c r="E4" s="12"/>
-      <c r="F4" s="13" t="s">
-        <v>14</v>
-      </c>
-      <c r="G4" s="13"/>
-      <c r="H4" s="13"/>
-      <c r="I4" s="13"/>
-      <c r="J4" s="13"/>
-      <c r="K4" s="13"/>
-      <c r="L4" s="14" t="s">
+      <c r="A4" s="9" t="s">
+        <v>1</v>
+      </c>
+      <c r="B4" s="9"/>
+      <c r="C4" s="9"/>
+      <c r="D4" s="9"/>
+      <c r="E4" s="9"/>
+      <c r="F4" s="10" t="s">
+        <v>13</v>
+      </c>
+      <c r="G4" s="10"/>
+      <c r="H4" s="10"/>
+      <c r="I4" s="10"/>
+      <c r="J4" s="10"/>
+      <c r="K4" s="10"/>
+      <c r="L4" s="11" t="s">
+        <v>15</v>
+      </c>
+      <c r="M4" s="11"/>
+      <c r="N4" s="11"/>
+      <c r="O4" s="11"/>
+      <c r="P4" s="11"/>
+      <c r="Q4" s="11"/>
+      <c r="R4" s="12" t="s">
         <v>16</v>
       </c>
-      <c r="M4" s="14"/>
-      <c r="N4" s="14"/>
-      <c r="O4" s="14"/>
-      <c r="P4" s="14"/>
-      <c r="Q4" s="14"/>
-      <c r="R4" s="11" t="s">
+      <c r="S4" s="12"/>
+      <c r="T4" s="12"/>
+      <c r="U4" s="12"/>
+      <c r="V4" s="12"/>
+      <c r="W4" s="12"/>
+      <c r="X4" s="12"/>
+      <c r="Y4" s="12"/>
+      <c r="Z4" s="12"/>
+      <c r="AA4" s="12"/>
+      <c r="AB4" s="12"/>
+      <c r="AC4" s="12"/>
+      <c r="AD4" s="12"/>
+      <c r="AE4" s="12"/>
+      <c r="AF4" s="12"/>
+      <c r="AG4" s="12"/>
+      <c r="AH4" s="12"/>
+      <c r="AI4" s="12"/>
+      <c r="AJ4" s="11" t="s">
         <v>17</v>
       </c>
-      <c r="S4" s="11"/>
-      <c r="T4" s="11"/>
-      <c r="U4" s="11"/>
-      <c r="V4" s="11"/>
-      <c r="W4" s="11"/>
-      <c r="X4" s="11"/>
-      <c r="Y4" s="11"/>
-      <c r="Z4" s="11"/>
-      <c r="AA4" s="11"/>
-      <c r="AB4" s="11"/>
-      <c r="AC4" s="11"/>
-      <c r="AD4" s="11"/>
-      <c r="AE4" s="11"/>
-      <c r="AF4" s="11"/>
-      <c r="AG4" s="11"/>
-      <c r="AH4" s="11"/>
-      <c r="AI4" s="11"/>
-      <c r="AJ4" s="14" t="s">
-        <v>18</v>
-      </c>
-      <c r="AK4" s="14"/>
-      <c r="AL4" s="14"/>
-      <c r="AM4" s="14"/>
-      <c r="AN4" s="14"/>
-      <c r="AO4" s="14"/>
+      <c r="AK4" s="11"/>
+      <c r="AL4" s="11"/>
+      <c r="AM4" s="11"/>
+      <c r="AN4" s="11"/>
+      <c r="AO4" s="11"/>
     </row>
     <row r="5" spans="1:41" s="7" customFormat="1" ht="45" customHeight="1" x14ac:dyDescent="0.3">
-      <c r="A5" s="9"/>
-      <c r="B5" s="9" t="s">
+      <c r="A5" s="13"/>
+      <c r="B5" s="13" t="s">
+        <v>2</v>
+      </c>
+      <c r="C5" s="13" t="s">
         <v>3</v>
       </c>
-      <c r="C5" s="9" t="s">
+      <c r="D5" s="13" t="s">
         <v>4</v>
       </c>
-      <c r="D5" s="9" t="s">
+      <c r="E5" s="13" t="s">
         <v>5</v>
       </c>
-      <c r="E5" s="9" t="s">
+      <c r="F5" s="14" t="s">
         <v>6</v>
       </c>
-      <c r="F5" s="10" t="s">
+      <c r="G5" s="14" t="s">
         <v>7</v>
       </c>
-      <c r="G5" s="10" t="s">
+      <c r="H5" s="14" t="s">
         <v>8</v>
       </c>
-      <c r="H5" s="10" t="s">
+      <c r="I5" s="14" t="s">
         <v>9</v>
       </c>
-      <c r="I5" s="10" t="s">
+      <c r="J5" s="13" t="s">
         <v>10</v>
       </c>
-      <c r="J5" s="9" t="s">
+      <c r="K5" s="14" t="s">
         <v>11</v>
       </c>
-      <c r="K5" s="10" t="s">
-        <v>12</v>
-      </c>
-      <c r="L5" s="9" t="s">
+      <c r="L5" s="13" t="s">
+        <v>18</v>
+      </c>
+      <c r="M5" s="13" t="s">
         <v>19</v>
       </c>
-      <c r="M5" s="9" t="s">
+      <c r="N5" s="13" t="s">
         <v>20</v>
       </c>
-      <c r="N5" s="9" t="s">
+      <c r="O5" s="13" t="s">
         <v>21</v>
       </c>
-      <c r="O5" s="9" t="s">
+      <c r="P5" s="13" t="s">
         <v>22</v>
       </c>
-      <c r="P5" s="9" t="s">
+      <c r="Q5" s="13" t="s">
         <v>23</v>
       </c>
-      <c r="Q5" s="9" t="s">
+      <c r="R5" s="12" t="s">
         <v>24</v>
       </c>
-      <c r="R5" s="11" t="s">
+      <c r="S5" s="12"/>
+      <c r="T5" s="12"/>
+      <c r="U5" s="12"/>
+      <c r="V5" s="12"/>
+      <c r="W5" s="12"/>
+      <c r="X5" s="12" t="s">
         <v>25</v>
       </c>
-      <c r="S5" s="11"/>
-      <c r="T5" s="11"/>
-      <c r="U5" s="11"/>
-      <c r="V5" s="11"/>
-      <c r="W5" s="11"/>
-      <c r="X5" s="11" t="s">
+      <c r="Y5" s="12"/>
+      <c r="Z5" s="12"/>
+      <c r="AA5" s="12"/>
+      <c r="AB5" s="12"/>
+      <c r="AC5" s="12"/>
+      <c r="AD5" s="12" t="s">
         <v>26</v>
       </c>
-      <c r="Y5" s="11"/>
-      <c r="Z5" s="11"/>
-      <c r="AA5" s="11"/>
-      <c r="AB5" s="11"/>
-      <c r="AC5" s="11"/>
-      <c r="AD5" s="11" t="s">
+      <c r="AE5" s="12"/>
+      <c r="AF5" s="12"/>
+      <c r="AG5" s="12"/>
+      <c r="AH5" s="12"/>
+      <c r="AI5" s="12"/>
+      <c r="AJ5" s="13" t="s">
         <v>27</v>
       </c>
-      <c r="AE5" s="11"/>
-      <c r="AF5" s="11"/>
-      <c r="AG5" s="11"/>
-      <c r="AH5" s="11"/>
-      <c r="AI5" s="11"/>
-      <c r="AJ5" s="9" t="s">
+      <c r="AK5" s="13" t="s">
         <v>28</v>
       </c>
-      <c r="AK5" s="9" t="s">
+      <c r="AL5" s="13" t="s">
         <v>29</v>
       </c>
-      <c r="AL5" s="9" t="s">
+      <c r="AM5" s="13" t="s">
         <v>30</v>
       </c>
-      <c r="AM5" s="9" t="s">
+      <c r="AN5" s="13" t="s">
         <v>31</v>
       </c>
-      <c r="AN5" s="9" t="s">
+      <c r="AO5" s="13" t="s">
         <v>32</v>
-      </c>
-      <c r="AO5" s="9" t="s">
-        <v>33</v>
       </c>
     </row>
     <row r="6" spans="1:41" s="8" customFormat="1" ht="45" x14ac:dyDescent="0.2">
-      <c r="A6" s="9"/>
-      <c r="B6" s="9"/>
-      <c r="C6" s="9"/>
-      <c r="D6" s="9"/>
-      <c r="E6" s="9"/>
-      <c r="F6" s="10"/>
-      <c r="G6" s="10"/>
-      <c r="H6" s="10"/>
-      <c r="I6" s="10"/>
-      <c r="J6" s="9"/>
-      <c r="K6" s="10"/>
-      <c r="L6" s="9" t="s">
+      <c r="A6" s="13"/>
+      <c r="B6" s="13"/>
+      <c r="C6" s="13"/>
+      <c r="D6" s="13"/>
+      <c r="E6" s="13"/>
+      <c r="F6" s="14"/>
+      <c r="G6" s="14"/>
+      <c r="H6" s="14"/>
+      <c r="I6" s="14"/>
+      <c r="J6" s="13"/>
+      <c r="K6" s="14"/>
+      <c r="L6" s="13" t="s">
+        <v>18</v>
+      </c>
+      <c r="M6" s="13" t="s">
         <v>19</v>
       </c>
-      <c r="M6" s="9" t="s">
+      <c r="N6" s="13" t="s">
         <v>20</v>
       </c>
-      <c r="N6" s="9" t="s">
+      <c r="O6" s="13" t="s">
         <v>21</v>
       </c>
-      <c r="O6" s="9" t="s">
+      <c r="P6" s="13" t="s">
         <v>22</v>
       </c>
-      <c r="P6" s="9" t="s">
+      <c r="Q6" s="13" t="s">
         <v>23</v>
       </c>
-      <c r="Q6" s="9" t="s">
-        <v>24</v>
-      </c>
       <c r="R6" s="6" t="s">
+        <v>33</v>
+      </c>
+      <c r="S6" s="6" t="s">
         <v>34</v>
       </c>
-      <c r="S6" s="6" t="s">
+      <c r="T6" s="6" t="s">
         <v>35</v>
       </c>
-      <c r="T6" s="6" t="s">
+      <c r="U6" s="6" t="s">
         <v>36</v>
       </c>
-      <c r="U6" s="6" t="s">
+      <c r="V6" s="6" t="s">
         <v>37</v>
       </c>
-      <c r="V6" s="6" t="s">
+      <c r="W6" s="6" t="s">
         <v>38</v>
       </c>
-      <c r="W6" s="6" t="s">
+      <c r="X6" s="6" t="s">
         <v>39</v>
       </c>
-      <c r="X6" s="6" t="s">
+      <c r="Y6" s="6" t="s">
         <v>40</v>
       </c>
-      <c r="Y6" s="6" t="s">
+      <c r="Z6" s="6" t="s">
         <v>41</v>
       </c>
-      <c r="Z6" s="6" t="s">
+      <c r="AA6" s="6" t="s">
         <v>42</v>
       </c>
-      <c r="AA6" s="6" t="s">
+      <c r="AB6" s="6" t="s">
         <v>43</v>
       </c>
-      <c r="AB6" s="6" t="s">
+      <c r="AC6" s="6" t="s">
         <v>44</v>
       </c>
-      <c r="AC6" s="6" t="s">
+      <c r="AD6" s="6" t="s">
         <v>45</v>
       </c>
-      <c r="AD6" s="6" t="s">
+      <c r="AE6" s="6" t="s">
         <v>46</v>
       </c>
-      <c r="AE6" s="6" t="s">
+      <c r="AF6" s="6" t="s">
         <v>47</v>
       </c>
-      <c r="AF6" s="6" t="s">
+      <c r="AG6" s="6" t="s">
         <v>48</v>
       </c>
-      <c r="AG6" s="6" t="s">
+      <c r="AH6" s="6" t="s">
         <v>49</v>
       </c>
-      <c r="AH6" s="6" t="s">
+      <c r="AI6" s="6" t="s">
         <v>50</v>
       </c>
-      <c r="AI6" s="6" t="s">
-        <v>51</v>
-      </c>
-      <c r="AJ6" s="9" t="s">
+      <c r="AJ6" s="13" t="s">
+        <v>18</v>
+      </c>
+      <c r="AK6" s="13" t="s">
         <v>19</v>
       </c>
-      <c r="AK6" s="9" t="s">
-        <v>20</v>
-      </c>
-      <c r="AL6" s="9" t="s">
+      <c r="AL6" s="13" t="s">
+        <v>18</v>
+      </c>
+      <c r="AM6" s="13" t="s">
         <v>19</v>
       </c>
-      <c r="AM6" s="9" t="s">
-        <v>20</v>
-      </c>
-      <c r="AN6" s="9" t="s">
+      <c r="AN6" s="13" t="s">
+        <v>18</v>
+      </c>
+      <c r="AO6" s="13" t="s">
         <v>19</v>
-      </c>
-      <c r="AO6" s="9" t="s">
-        <v>20</v>
       </c>
     </row>
     <row r="7" spans="1:41" ht="15" x14ac:dyDescent="0.2">
       <c r="A7" s="8" t="s">
-        <v>15</v>
+        <v>14</v>
       </c>
     </row>
     <row r="10" spans="1:41" ht="15" customHeight="1" x14ac:dyDescent="0.2"/>
   </sheetData>
   <mergeCells count="31">
-    <mergeCell ref="A4:E4"/>
-    <mergeCell ref="F4:K4"/>
-    <mergeCell ref="L4:Q4"/>
-    <mergeCell ref="R4:AI4"/>
-    <mergeCell ref="AJ4:AO4"/>
-    <mergeCell ref="AM5:AM6"/>
-    <mergeCell ref="AN5:AN6"/>
-    <mergeCell ref="AO5:AO6"/>
-    <mergeCell ref="O5:O6"/>
-    <mergeCell ref="P5:P6"/>
-    <mergeCell ref="Q5:Q6"/>
-    <mergeCell ref="R5:W5"/>
-    <mergeCell ref="X5:AC5"/>
-    <mergeCell ref="AD5:AI5"/>
-    <mergeCell ref="AJ5:AJ6"/>
-    <mergeCell ref="AK5:AK6"/>
-    <mergeCell ref="AL5:AL6"/>
     <mergeCell ref="L5:L6"/>
     <mergeCell ref="M5:M6"/>
     <mergeCell ref="N5:N6"/>
@@ -983,29 +966,29 @@
     <mergeCell ref="I5:I6"/>
     <mergeCell ref="J5:J6"/>
     <mergeCell ref="K5:K6"/>
+    <mergeCell ref="AM5:AM6"/>
+    <mergeCell ref="AN5:AN6"/>
+    <mergeCell ref="AO5:AO6"/>
+    <mergeCell ref="O5:O6"/>
+    <mergeCell ref="P5:P6"/>
+    <mergeCell ref="Q5:Q6"/>
+    <mergeCell ref="R5:W5"/>
+    <mergeCell ref="X5:AC5"/>
+    <mergeCell ref="AD5:AI5"/>
+    <mergeCell ref="AJ5:AJ6"/>
+    <mergeCell ref="AK5:AK6"/>
+    <mergeCell ref="AL5:AL6"/>
+    <mergeCell ref="A4:E4"/>
+    <mergeCell ref="F4:K4"/>
+    <mergeCell ref="L4:Q4"/>
+    <mergeCell ref="R4:AI4"/>
+    <mergeCell ref="AJ4:AO4"/>
   </mergeCells>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
 </worksheet>
 </file>
 
 <file path=customXml/item1.xml><?xml version="1.0" encoding="utf-8"?>
-<?mso-contentType ?>
-<FormTemplates xmlns="http://schemas.microsoft.com/sharepoint/v3/contenttype/forms">
-  <Display>DocumentLibraryForm</Display>
-  <Edit>DocumentLibraryForm</Edit>
-  <New>DocumentLibraryForm</New>
-</FormTemplates>
-</file>
-
-<file path=customXml/item2.xml><?xml version="1.0" encoding="utf-8"?>
-<p:properties xmlns:p="http://schemas.microsoft.com/office/2006/metadata/properties" xmlns:xsi="http://www.w3.org/2001/XMLSchema-instance" xmlns:pc="http://schemas.microsoft.com/office/infopath/2007/PartnerControls">
-  <documentManagement>
-    <_activity xmlns="9c5e610e-28db-44df-ba41-c446aaffe434" xsi:nil="true"/>
-  </documentManagement>
-</p:properties>
-</file>
-
-<file path=customXml/item3.xml><?xml version="1.0" encoding="utf-8"?>
 <ct:contentTypeSchema xmlns:ct="http://schemas.microsoft.com/office/2006/metadata/contentType" xmlns:ma="http://schemas.microsoft.com/office/2006/metadata/properties/metaAttributes" ct:_="" ma:_="" ma:contentTypeName="Document" ma:contentTypeID="0x010100E2AA525DA2F333468273E03D890440D6" ma:contentTypeVersion="14" ma:contentTypeDescription="Create a new document." ma:contentTypeScope="" ma:versionID="a0f9360bda923dd7fb76d00a461df4cd">
   <xsd:schema xmlns:xsd="http://www.w3.org/2001/XMLSchema" xmlns:xs="http://www.w3.org/2001/XMLSchema" xmlns:p="http://schemas.microsoft.com/office/2006/metadata/properties" xmlns:ns3="9c5e610e-28db-44df-ba41-c446aaffe434" xmlns:ns4="e78f2374-cb69-45b5-92b0-6a1f828922e7" targetNamespace="http://schemas.microsoft.com/office/2006/metadata/properties" ma:root="true" ma:fieldsID="e929c21602ddc082d402d6da66c8cbef" ns3:_="" ns4:_="">
     <xsd:import namespace="9c5e610e-28db-44df-ba41-c446aaffe434"/>
@@ -1232,10 +1215,38 @@
 </ct:contentTypeSchema>
 </file>
 
+<file path=customXml/item2.xml><?xml version="1.0" encoding="utf-8"?>
+<p:properties xmlns:p="http://schemas.microsoft.com/office/2006/metadata/properties" xmlns:xsi="http://www.w3.org/2001/XMLSchema-instance" xmlns:pc="http://schemas.microsoft.com/office/infopath/2007/PartnerControls">
+  <documentManagement>
+    <_activity xmlns="9c5e610e-28db-44df-ba41-c446aaffe434" xsi:nil="true"/>
+  </documentManagement>
+</p:properties>
+</file>
+
+<file path=customXml/item3.xml><?xml version="1.0" encoding="utf-8"?>
+<?mso-contentType ?>
+<FormTemplates xmlns="http://schemas.microsoft.com/sharepoint/v3/contenttype/forms">
+  <Display>DocumentLibraryForm</Display>
+  <Edit>DocumentLibraryForm</Edit>
+  <New>DocumentLibraryForm</New>
+</FormTemplates>
+</file>
+
 <file path=customXml/itemProps1.xml><?xml version="1.0" encoding="utf-8"?>
-<ds:datastoreItem xmlns:ds="http://schemas.openxmlformats.org/officeDocument/2006/customXml" ds:itemID="{37FFED95-5729-4606-80C4-D23BA0F5A716}">
+<ds:datastoreItem xmlns:ds="http://schemas.openxmlformats.org/officeDocument/2006/customXml" ds:itemID="{9B070AD9-465D-489D-95B7-FF09653BA1CD}">
   <ds:schemaRefs>
-    <ds:schemaRef ds:uri="http://schemas.microsoft.com/sharepoint/v3/contenttype/forms"/>
+    <ds:schemaRef ds:uri="http://schemas.microsoft.com/office/2006/metadata/contentType"/>
+    <ds:schemaRef ds:uri="http://schemas.microsoft.com/office/2006/metadata/properties/metaAttributes"/>
+    <ds:schemaRef ds:uri="http://www.w3.org/2001/XMLSchema"/>
+    <ds:schemaRef ds:uri="http://schemas.microsoft.com/office/2006/metadata/properties"/>
+    <ds:schemaRef ds:uri="9c5e610e-28db-44df-ba41-c446aaffe434"/>
+    <ds:schemaRef ds:uri="e78f2374-cb69-45b5-92b0-6a1f828922e7"/>
+    <ds:schemaRef ds:uri="http://schemas.microsoft.com/office/2006/documentManagement/types"/>
+    <ds:schemaRef ds:uri="http://schemas.microsoft.com/office/infopath/2007/PartnerControls"/>
+    <ds:schemaRef ds:uri="http://schemas.openxmlformats.org/package/2006/metadata/core-properties"/>
+    <ds:schemaRef ds:uri="http://purl.org/dc/elements/1.1/"/>
+    <ds:schemaRef ds:uri="http://purl.org/dc/terms/"/>
+    <ds:schemaRef ds:uri="http://schemas.microsoft.com/internal/obd"/>
   </ds:schemaRefs>
 </ds:datastoreItem>
 </file>
@@ -1258,20 +1269,9 @@
 </file>
 
 <file path=customXml/itemProps3.xml><?xml version="1.0" encoding="utf-8"?>
-<ds:datastoreItem xmlns:ds="http://schemas.openxmlformats.org/officeDocument/2006/customXml" ds:itemID="{9B070AD9-465D-489D-95B7-FF09653BA1CD}">
+<ds:datastoreItem xmlns:ds="http://schemas.openxmlformats.org/officeDocument/2006/customXml" ds:itemID="{37FFED95-5729-4606-80C4-D23BA0F5A716}">
   <ds:schemaRefs>
-    <ds:schemaRef ds:uri="http://schemas.microsoft.com/office/2006/metadata/contentType"/>
-    <ds:schemaRef ds:uri="http://schemas.microsoft.com/office/2006/metadata/properties/metaAttributes"/>
-    <ds:schemaRef ds:uri="http://www.w3.org/2001/XMLSchema"/>
-    <ds:schemaRef ds:uri="http://schemas.microsoft.com/office/2006/metadata/properties"/>
-    <ds:schemaRef ds:uri="9c5e610e-28db-44df-ba41-c446aaffe434"/>
-    <ds:schemaRef ds:uri="e78f2374-cb69-45b5-92b0-6a1f828922e7"/>
-    <ds:schemaRef ds:uri="http://schemas.microsoft.com/office/2006/documentManagement/types"/>
-    <ds:schemaRef ds:uri="http://schemas.microsoft.com/office/infopath/2007/PartnerControls"/>
-    <ds:schemaRef ds:uri="http://schemas.openxmlformats.org/package/2006/metadata/core-properties"/>
-    <ds:schemaRef ds:uri="http://purl.org/dc/elements/1.1/"/>
-    <ds:schemaRef ds:uri="http://purl.org/dc/terms/"/>
-    <ds:schemaRef ds:uri="http://schemas.microsoft.com/internal/obd"/>
+    <ds:schemaRef ds:uri="http://schemas.microsoft.com/sharepoint/v3/contenttype/forms"/>
   </ds:schemaRefs>
 </ds:datastoreItem>
 </file>
</xml_diff>